<commit_message>
fixing unit issues throughout many files
</commit_message>
<xml_diff>
--- a/data/raw/51293-2025-01-childnutrition.xlsx
+++ b/data/raw/51293-2025-01-childnutrition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\cbo.gov\Shares\BAD\BAD_DATA\Shared\Supplemental Data Tables\2025\January 2025  baseline\2-First Drafts January 2025 Baseline\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/481781ca8254c580/Desktop/OneDrive Desktop files/Sandboxes/Data_friendly_CBO_Baseline_Detail/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1A0B18-B167-41BC-8B17-8336F2F3CC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EF1A0B18-B167-41BC-8B17-8336F2F3CC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1451B521-13CC-4B5C-A2ED-2B8ED15C0B4F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FDA63628-CA73-42CC-9ACE-5FF0AB6A639D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{FDA63628-CA73-42CC-9ACE-5FF0AB6A639D}"/>
   </bookViews>
   <sheets>
     <sheet name="Child Nutrition_01-2025 (2)" sheetId="1" r:id="rId1"/>
@@ -549,7 +549,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
     <numFmt numFmtId="165" formatCode="###.\ "/>
@@ -876,7 +876,9 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{B638431B-506A-48EC-B07B-5F6CA71EA28F}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -3549,6 +3551,9 @@
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Current Assump."/>
       <sheetName val="Housing"/>
@@ -4204,19 +4209,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P77"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.3046875" defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.69140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" width="40.7109375" style="1" customWidth="1"/>
-    <col min="4" max="14" width="8.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="11.85546875" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.28515625" style="1"/>
+    <col min="3" max="3" width="40.69140625" style="1" customWidth="1"/>
+    <col min="4" max="14" width="8.69140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.15234375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="11.84375" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.3046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3" t="s">
@@ -4238,7 +4243,7 @@
       <c r="O2" s="63"/>
       <c r="P2" s="63"/>
     </row>
-    <row r="3" spans="1:16" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="17.600000000000001" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
@@ -4258,7 +4263,7 @@
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
     </row>
-    <row r="4" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="7" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -4276,7 +4281,7 @@
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
     </row>
-    <row r="5" spans="1:16" s="8" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" s="8" customFormat="1" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="A5" s="58"/>
       <c r="B5" s="58"/>
       <c r="C5" s="58"/>
@@ -4294,7 +4299,7 @@
       <c r="O5" s="60"/>
       <c r="P5" s="60"/>
     </row>
-    <row r="6" spans="1:16" s="8" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" s="8" customFormat="1" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="A6" s="64" t="s">
         <v>3</v>
       </c>
@@ -4314,7 +4319,7 @@
       <c r="O6" s="60"/>
       <c r="P6" s="60"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="10"/>
       <c r="C7" s="11"/>
@@ -4336,7 +4341,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
       <c r="C8" s="16"/>
@@ -4380,7 +4385,7 @@
         <v>2035</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19"/>
       <c r="B9" s="10"/>
       <c r="C9" s="11"/>
@@ -4398,7 +4403,7 @@
       <c r="O9" s="13"/>
       <c r="P9" s="13"/>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="21" t="s">
         <v>5</v>
       </c>
@@ -4422,7 +4427,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
         <v>7</v>
       </c>
@@ -4442,7 +4447,7 @@
       <c r="O11" s="24"/>
       <c r="P11" s="24"/>
     </row>
-    <row r="12" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="7" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="25"/>
       <c r="B12" s="9"/>
       <c r="C12" s="22"/>
@@ -4460,7 +4465,7 @@
       <c r="O12" s="26"/>
       <c r="P12" s="26"/>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="22" t="s">
         <v>8</v>
       </c>
@@ -4506,7 +4511,7 @@
         <v>429343</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="22"/>
       <c r="B14" s="22"/>
       <c r="C14" s="22"/>
@@ -4524,7 +4529,7 @@
       <c r="O14" s="26"/>
       <c r="P14" s="26"/>
     </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="22" t="s">
         <v>9</v>
       </c>
@@ -4570,7 +4575,7 @@
         <v>426724</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="22"/>
       <c r="B16" s="22"/>
       <c r="C16" s="22"/>
@@ -4588,7 +4593,7 @@
       <c r="O16" s="26"/>
       <c r="P16" s="26"/>
     </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="30" t="s">
         <v>10</v>
       </c>
@@ -4608,7 +4613,7 @@
       <c r="O17" s="26"/>
       <c r="P17" s="26"/>
     </row>
-    <row r="18" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="30"/>
       <c r="B18" s="30"/>
       <c r="C18" s="30"/>
@@ -4626,7 +4631,7 @@
       <c r="O18" s="26"/>
       <c r="P18" s="26"/>
     </row>
-    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="32" t="s">
         <v>11</v>
       </c>
@@ -4646,7 +4651,7 @@
       <c r="O19" s="26"/>
       <c r="P19" s="26"/>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="30"/>
       <c r="B20" s="33" t="s">
         <v>12</v>
@@ -4692,7 +4697,7 @@
         <v>224247</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="30"/>
       <c r="B21" s="35" t="s">
         <v>9</v>
@@ -4738,7 +4743,7 @@
         <v>222863</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="30"/>
       <c r="B22" s="30"/>
       <c r="C22" s="30"/>
@@ -4756,7 +4761,7 @@
       <c r="O22" s="26"/>
       <c r="P22" s="26"/>
     </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="32" t="s">
         <v>13</v>
       </c>
@@ -4776,7 +4781,7 @@
       <c r="O23" s="26"/>
       <c r="P23" s="26"/>
     </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="30"/>
       <c r="B24" s="33" t="s">
         <v>8</v>
@@ -4822,7 +4827,7 @@
         <v>78301</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="30"/>
       <c r="B25" s="35" t="s">
         <v>9</v>
@@ -4868,7 +4873,7 @@
         <v>77822</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="30"/>
       <c r="B26" s="30"/>
       <c r="C26" s="30"/>
@@ -4886,7 +4891,7 @@
       <c r="O26" s="26"/>
       <c r="P26" s="26"/>
     </row>
-    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="32" t="s">
         <v>14</v>
       </c>
@@ -4906,7 +4911,7 @@
       <c r="O27" s="26"/>
       <c r="P27" s="26"/>
     </row>
-    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="30"/>
       <c r="B28" s="33" t="s">
         <v>8</v>
@@ -4952,7 +4957,7 @@
         <v>55098</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="30"/>
       <c r="B29" s="35" t="s">
         <v>9</v>
@@ -4998,7 +5003,7 @@
         <v>54764</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="30"/>
       <c r="B30" s="30"/>
       <c r="C30" s="30"/>
@@ -5016,7 +5021,7 @@
       <c r="O30" s="26"/>
       <c r="P30" s="26"/>
     </row>
-    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="32" t="s">
         <v>15</v>
       </c>
@@ -5036,7 +5041,7 @@
       <c r="O31" s="26"/>
       <c r="P31" s="26"/>
     </row>
-    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="30"/>
       <c r="B32" s="33" t="s">
         <v>8</v>
@@ -5082,7 +5087,7 @@
         <v>27751</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="30"/>
       <c r="B33" s="35" t="s">
         <v>9</v>
@@ -5128,7 +5133,7 @@
         <v>27582</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="30"/>
       <c r="B34" s="35"/>
       <c r="C34" s="30"/>
@@ -5146,7 +5151,7 @@
       <c r="O34" s="26"/>
       <c r="P34" s="26"/>
     </row>
-    <row r="35" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="32" t="s">
         <v>16</v>
       </c>
@@ -5166,7 +5171,7 @@
       <c r="O35" s="26"/>
       <c r="P35" s="26"/>
     </row>
-    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="32"/>
       <c r="B36" s="33" t="s">
         <v>8</v>
@@ -5212,7 +5217,7 @@
         <v>36392</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="32"/>
       <c r="B37" s="35" t="s">
         <v>9</v>
@@ -5258,7 +5263,7 @@
         <v>36169</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="32"/>
       <c r="B38" s="30"/>
       <c r="C38" s="30"/>
@@ -5276,7 +5281,7 @@
       <c r="O38" s="26"/>
       <c r="P38" s="26"/>
     </row>
-    <row r="39" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="32" t="s">
         <v>17</v>
       </c>
@@ -5296,7 +5301,7 @@
       <c r="O39" s="26"/>
       <c r="P39" s="26"/>
     </row>
-    <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="30"/>
       <c r="B40" s="33" t="s">
         <v>8</v>
@@ -5342,7 +5347,7 @@
         <v>4944</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="30"/>
       <c r="B41" s="35" t="s">
         <v>9</v>
@@ -5388,7 +5393,7 @@
         <v>4914</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="30"/>
       <c r="B42" s="35"/>
       <c r="C42" s="30"/>
@@ -5406,7 +5411,7 @@
       <c r="O42" s="26"/>
       <c r="P42" s="26"/>
     </row>
-    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="32" t="s">
         <v>18</v>
       </c>
@@ -5426,7 +5431,7 @@
       <c r="O43" s="26"/>
       <c r="P43" s="26"/>
     </row>
-    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="30"/>
       <c r="B44" s="33" t="s">
         <v>8</v>
@@ -5472,7 +5477,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="30"/>
       <c r="B45" s="35" t="s">
         <v>9</v>
@@ -5518,7 +5523,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="7.35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" ht="7.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="36"/>
       <c r="B46" s="37"/>
       <c r="C46" s="38"/>
@@ -5536,7 +5541,7 @@
       <c r="O46" s="40"/>
       <c r="P46" s="40"/>
     </row>
-    <row r="47" spans="1:16" ht="7.35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" ht="7.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="9"/>
       <c r="B47" s="41"/>
       <c r="C47" s="22"/>
@@ -5554,7 +5559,7 @@
       <c r="O47" s="22"/>
       <c r="P47" s="22"/>
     </row>
-    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="42" t="s">
         <v>19</v>
       </c>
@@ -5574,7 +5579,7 @@
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
     </row>
-    <row r="49" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>20</v>
       </c>
@@ -5594,7 +5599,7 @@
       <c r="O49" s="22"/>
       <c r="P49" s="22"/>
     </row>
-    <row r="50" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" ht="7" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="42"/>
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
@@ -5612,7 +5617,7 @@
       <c r="O50" s="22"/>
       <c r="P50" s="22"/>
     </row>
-    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -5650,7 +5655,7 @@
       <c r="O51" s="22"/>
       <c r="P51" s="22"/>
     </row>
-    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="42"/>
       <c r="B52" s="9"/>
       <c r="C52" s="23" t="s">
@@ -5690,7 +5695,7 @@
       <c r="O52" s="22"/>
       <c r="P52" s="22"/>
     </row>
-    <row r="53" spans="1:16" ht="2.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="36"/>
       <c r="B53" s="37"/>
       <c r="C53" s="38"/>
@@ -5708,7 +5713,7 @@
       <c r="O53" s="38"/>
       <c r="P53" s="38"/>
     </row>
-    <row r="54" spans="1:16" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="9"/>
       <c r="B54" s="41"/>
       <c r="C54" s="22"/>
@@ -5726,7 +5731,7 @@
       <c r="O54" s="46"/>
       <c r="P54" s="46"/>
     </row>
-    <row r="55" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="47" t="s">
         <v>22</v>
       </c>
@@ -5746,7 +5751,7 @@
       <c r="O55" s="50"/>
       <c r="P55" s="50"/>
     </row>
-    <row r="56" spans="1:16" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" ht="4.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="47"/>
       <c r="B56" s="48"/>
       <c r="C56" s="49"/>
@@ -5764,7 +5769,7 @@
       <c r="O56" s="50"/>
       <c r="P56" s="50"/>
     </row>
-    <row r="57" spans="1:16" s="52" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" s="52" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A57" s="51" t="s">
         <v>23</v>
       </c>
@@ -5786,7 +5791,7 @@
       <c r="O57" s="65"/>
       <c r="P57" s="65"/>
     </row>
-    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="51"/>
       <c r="B58" s="65"/>
       <c r="C58" s="65"/>
@@ -5804,7 +5809,7 @@
       <c r="O58" s="65"/>
       <c r="P58" s="65"/>
     </row>
-    <row r="59" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="51"/>
       <c r="B59" s="65"/>
       <c r="C59" s="65"/>
@@ -5822,7 +5827,7 @@
       <c r="O59" s="65"/>
       <c r="P59" s="65"/>
     </row>
-    <row r="60" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="51"/>
       <c r="B60" s="65"/>
       <c r="C60" s="65"/>
@@ -5840,7 +5845,7 @@
       <c r="O60" s="65"/>
       <c r="P60" s="65"/>
     </row>
-    <row r="61" spans="1:16" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" ht="7" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="51"/>
       <c r="B61" s="65"/>
       <c r="C61" s="65"/>
@@ -5858,7 +5863,7 @@
       <c r="O61" s="65"/>
       <c r="P61" s="65"/>
     </row>
-    <row r="62" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D62" s="53"/>
       <c r="E62" s="53"/>
       <c r="F62" s="53"/>
@@ -5871,10 +5876,10 @@
       <c r="M62" s="53"/>
       <c r="N62" s="53"/>
     </row>
-    <row r="63" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="65" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="66" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="54"/>
       <c r="B66" s="54"/>
       <c r="C66" s="55"/>
@@ -5892,7 +5897,7 @@
       <c r="O66" s="54"/>
       <c r="P66" s="54"/>
     </row>
-    <row r="67" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="54"/>
       <c r="B67" s="54"/>
       <c r="C67" s="57"/>
@@ -5910,7 +5915,7 @@
       <c r="O67" s="54"/>
       <c r="P67" s="54"/>
     </row>
-    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="54"/>
       <c r="B68" s="54"/>
       <c r="C68" s="57"/>
@@ -5928,7 +5933,7 @@
       <c r="O68" s="54"/>
       <c r="P68" s="54"/>
     </row>
-    <row r="69" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="54"/>
       <c r="B69" s="54"/>
       <c r="C69" s="54"/>
@@ -5946,8 +5951,8 @@
       <c r="O69" s="54"/>
       <c r="P69" s="54"/>
     </row>
-    <row r="70" spans="1:16" s="54" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:16" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" s="54" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="1:16" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="54"/>
       <c r="B71" s="54"/>
       <c r="C71" s="54"/>
@@ -5965,7 +5970,7 @@
       <c r="O71" s="54"/>
       <c r="P71" s="54"/>
     </row>
-    <row r="72" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="54"/>
       <c r="B72" s="54"/>
       <c r="C72" s="54"/>
@@ -5983,7 +5988,7 @@
       <c r="O72" s="54"/>
       <c r="P72" s="54"/>
     </row>
-    <row r="73" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="54"/>
       <c r="B73" s="54"/>
       <c r="C73" s="54"/>
@@ -6001,7 +6006,7 @@
       <c r="O73" s="54"/>
       <c r="P73" s="54"/>
     </row>
-    <row r="74" spans="1:16" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="54"/>
       <c r="B74" s="54"/>
       <c r="C74" s="54"/>
@@ -6019,7 +6024,7 @@
       <c r="O74" s="54"/>
       <c r="P74" s="54"/>
     </row>
-    <row r="75" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="54"/>
       <c r="B75" s="54"/>
       <c r="C75" s="54"/>
@@ -6037,7 +6042,7 @@
       <c r="O75" s="54"/>
       <c r="P75" s="54"/>
     </row>
-    <row r="76" spans="1:16" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" ht="13.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="54"/>
       <c r="B76" s="54"/>
       <c r="C76" s="54"/>
@@ -6055,7 +6060,7 @@
       <c r="O76" s="54"/>
       <c r="P76" s="54"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="54"/>
       <c r="B77" s="54"/>
       <c r="C77" s="54"/>

</xml_diff>